<commit_message>
cambios para el score incluyendo duración por horas
</commit_message>
<xml_diff>
--- a/Result/ILP_Results.xlsx
+++ b/Result/ILP_Results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W150"/>
+  <dimension ref="A1:AB150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,15 +531,40 @@
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
+          <t>score_por_h</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>score_hibrido</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>dur_bin</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>penal_bin</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>score_final</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
           <t>Asignados</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Real_Agendas</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
@@ -632,12 +657,29 @@
         <v>8937</v>
       </c>
       <c r="U2" t="n">
+        <v>1051.411764705882</v>
+      </c>
+      <c r="V2" t="n">
+        <v>5782.764705882353</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X2" t="n">
+        <v>0.9136964823116547</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>5781.851009400041</v>
+      </c>
+      <c r="Z2" t="n">
         <v>30</v>
       </c>
-      <c r="V2" t="n">
+      <c r="AA2" t="n">
         <v>30</v>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -730,12 +772,29 @@
         <v>8937</v>
       </c>
       <c r="U3" t="n">
+        <v>940.7368421052631</v>
+      </c>
+      <c r="V3" t="n">
+        <v>5738.494736842105</v>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X3" t="n">
+        <v>0.4636563680037474</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>5738.031080474101</v>
+      </c>
+      <c r="Z3" t="n">
         <v>30</v>
       </c>
-      <c r="V3" t="n">
+      <c r="AA3" t="n">
         <v>30</v>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="AB3" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -828,12 +887,29 @@
         <v>8678</v>
       </c>
       <c r="U4" t="n">
+        <v>1020.941176470588</v>
+      </c>
+      <c r="V4" t="n">
+        <v>5615.176470588235</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X4" t="n">
+        <v>0.9136964823116547</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>5614.262774105923</v>
+      </c>
+      <c r="Z4" t="n">
         <v>21</v>
       </c>
-      <c r="V4" t="n">
+      <c r="AA4" t="n">
         <v>21</v>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="AB4" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -926,12 +1002,29 @@
         <v>8557</v>
       </c>
       <c r="U5" t="n">
-        <v>15</v>
+        <v>950.7777777777778</v>
       </c>
       <c r="V5" t="n">
-        <v>15</v>
+        <v>5514.511111111111</v>
       </c>
       <c r="W5" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X5" t="n">
+        <v>0.4636563680037474</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>5514.047454743107</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB5" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -1024,12 +1117,29 @@
         <v>8557</v>
       </c>
       <c r="U6" t="n">
-        <v>15</v>
+        <v>950.7777777777778</v>
       </c>
       <c r="V6" t="n">
-        <v>15</v>
+        <v>5514.511111111111</v>
       </c>
       <c r="W6" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X6" t="n">
+        <v>0.4636563680037474</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>5514.047454743107</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB6" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -1122,12 +1232,29 @@
         <v>8557</v>
       </c>
       <c r="U7" t="n">
-        <v>15</v>
+        <v>1006.705882352941</v>
       </c>
       <c r="V7" t="n">
-        <v>15</v>
+        <v>5536.882352941177</v>
       </c>
       <c r="W7" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X7" t="n">
+        <v>0.9136964823116547</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>5535.968656458865</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB7" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -1220,12 +1347,29 @@
         <v>8557</v>
       </c>
       <c r="U8" t="n">
-        <v>15</v>
+        <v>1037.212121212121</v>
       </c>
       <c r="V8" t="n">
-        <v>15</v>
+        <v>5549.084848484848</v>
       </c>
       <c r="W8" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X8" t="n">
+        <v>0.9136964823116547</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>5548.171152002536</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB8" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -1318,12 +1462,29 @@
         <v>8557</v>
       </c>
       <c r="U9" t="n">
-        <v>15</v>
+        <v>1006.705882352941</v>
       </c>
       <c r="V9" t="n">
-        <v>15</v>
+        <v>5536.882352941177</v>
       </c>
       <c r="W9" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X9" t="n">
+        <v>0.9136964823116547</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>5535.968656458865</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB9" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -1416,12 +1577,29 @@
         <v>8557</v>
       </c>
       <c r="U10" t="n">
-        <v>15</v>
+        <v>1069.625</v>
       </c>
       <c r="V10" t="n">
-        <v>15</v>
+        <v>5562.05</v>
       </c>
       <c r="W10" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X10" t="n">
+        <v>0.9136964823116547</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>5561.136303517688</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB10" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -1514,12 +1692,29 @@
         <v>8557</v>
       </c>
       <c r="U11" t="n">
-        <v>15</v>
+        <v>1016.673267326733</v>
       </c>
       <c r="V11" t="n">
-        <v>15</v>
+        <v>5540.869306930693</v>
       </c>
       <c r="W11" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X11" t="n">
+        <v>0.9136964823116547</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>5539.955610448381</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB11" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -1612,12 +1807,29 @@
         <v>8506</v>
       </c>
       <c r="U12" t="n">
+        <v>1000.705882352941</v>
+      </c>
+      <c r="V12" t="n">
+        <v>5503.882352941176</v>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X12" t="n">
+        <v>0.9136964823116547</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>5502.968656458864</v>
+      </c>
+      <c r="Z12" t="n">
         <v>3</v>
       </c>
-      <c r="V12" t="n">
+      <c r="AA12" t="n">
         <v>3</v>
       </c>
-      <c r="W12" t="inlineStr">
+      <c r="AB12" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -1710,12 +1922,29 @@
         <v>8506</v>
       </c>
       <c r="U13" t="n">
-        <v>15</v>
+        <v>895.3684210526316</v>
       </c>
       <c r="V13" t="n">
-        <v>15</v>
+        <v>5461.747368421052</v>
       </c>
       <c r="W13" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X13" t="n">
+        <v>0.4636563680037474</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>5461.283712053048</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB13" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -1808,12 +2037,29 @@
         <v>8488</v>
       </c>
       <c r="U14" t="n">
-        <v>15</v>
+        <v>943.1111111111111</v>
       </c>
       <c r="V14" t="n">
-        <v>15</v>
+        <v>5470.044444444445</v>
       </c>
       <c r="W14" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X14" t="n">
+        <v>0.4636563680037474</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>5469.580788076441</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB14" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -1906,12 +2152,29 @@
         <v>8488</v>
       </c>
       <c r="U15" t="n">
-        <v>15</v>
+        <v>998.5882352941177</v>
       </c>
       <c r="V15" t="n">
-        <v>15</v>
+        <v>5492.235294117647</v>
       </c>
       <c r="W15" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X15" t="n">
+        <v>0.9136964823116547</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>5491.321597635335</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB15" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -2004,12 +2267,29 @@
         <v>8488</v>
       </c>
       <c r="U16" t="n">
-        <v>15</v>
+        <v>943.1111111111111</v>
       </c>
       <c r="V16" t="n">
-        <v>15</v>
+        <v>5470.044444444445</v>
       </c>
       <c r="W16" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X16" t="n">
+        <v>0.4636563680037474</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>5469.580788076441</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB16" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -2102,12 +2382,29 @@
         <v>8488</v>
       </c>
       <c r="U17" t="n">
-        <v>15</v>
+        <v>1028.848484848485</v>
       </c>
       <c r="V17" t="n">
-        <v>15</v>
+        <v>5504.339393939394</v>
       </c>
       <c r="W17" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X17" t="n">
+        <v>0.9136964823116547</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>5503.425697457082</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB17" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -2200,12 +2497,29 @@
         <v>8488</v>
       </c>
       <c r="U18" t="n">
+        <v>1050.061855670103</v>
+      </c>
+      <c r="V18" t="n">
+        <v>5512.824742268042</v>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X18" t="n">
+        <v>0.9136964823116547</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>5511.91104578573</v>
+      </c>
+      <c r="Z18" t="n">
         <v>9</v>
       </c>
-      <c r="V18" t="n">
+      <c r="AA18" t="n">
         <v>9</v>
       </c>
-      <c r="W18" t="inlineStr">
+      <c r="AB18" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -2298,12 +2612,29 @@
         <v>8488</v>
       </c>
       <c r="U19" t="n">
-        <v>15</v>
+        <v>1028.848484848485</v>
       </c>
       <c r="V19" t="n">
-        <v>15</v>
+        <v>5504.339393939394</v>
       </c>
       <c r="W19" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X19" t="n">
+        <v>0.9136964823116547</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>5503.425697457082</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB19" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -2396,12 +2727,29 @@
         <v>8488</v>
       </c>
       <c r="U20" t="n">
-        <v>15</v>
+        <v>1061</v>
       </c>
       <c r="V20" t="n">
-        <v>15</v>
+        <v>5517.2</v>
       </c>
       <c r="W20" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X20" t="n">
+        <v>0.9136964823116547</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>5516.286303517688</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB20" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -2494,12 +2842,29 @@
         <v>8436</v>
       </c>
       <c r="U21" t="n">
-        <v>15</v>
+        <v>937.3333333333334</v>
       </c>
       <c r="V21" t="n">
-        <v>15</v>
+        <v>5436.533333333333</v>
       </c>
       <c r="W21" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X21" t="n">
+        <v>0.4636563680037474</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>5436.069676965329</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB21" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -2592,12 +2957,29 @@
         <v>8378</v>
       </c>
       <c r="U22" t="n">
-        <v>15</v>
+        <v>985.6470588235294</v>
       </c>
       <c r="V22" t="n">
-        <v>15</v>
+        <v>5421.058823529412</v>
       </c>
       <c r="W22" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X22" t="n">
+        <v>0.9136964823116547</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>5420.1451270471</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB22" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -2690,12 +3072,29 @@
         <v>8378</v>
       </c>
       <c r="U23" t="n">
-        <v>15</v>
+        <v>1047.25</v>
       </c>
       <c r="V23" t="n">
-        <v>15</v>
+        <v>5445.7</v>
       </c>
       <c r="W23" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X23" t="n">
+        <v>0.9136964823116547</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>5444.786303517688</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB23" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -2788,12 +3187,29 @@
         <v>8047</v>
       </c>
       <c r="U24" t="n">
-        <v>15</v>
+        <v>946.7058823529412</v>
       </c>
       <c r="V24" t="n">
-        <v>15</v>
+        <v>5206.882352941177</v>
       </c>
       <c r="W24" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X24" t="n">
+        <v>0.9136964823116547</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>5205.968656458865</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB24" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -2886,12 +3302,29 @@
         <v>8047</v>
       </c>
       <c r="U25" t="n">
-        <v>15</v>
+        <v>1005.875</v>
       </c>
       <c r="V25" t="n">
-        <v>15</v>
+        <v>5230.55</v>
       </c>
       <c r="W25" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X25" t="n">
+        <v>0.9136964823116547</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>5229.636303517688</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA25" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB25" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -2984,12 +3417,29 @@
         <v>8047</v>
       </c>
       <c r="U26" t="n">
-        <v>15</v>
+        <v>946.7058823529412</v>
       </c>
       <c r="V26" t="n">
-        <v>15</v>
+        <v>5206.882352941177</v>
       </c>
       <c r="W26" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X26" t="n">
+        <v>0.9136964823116547</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>5205.968656458865</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB26" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -3082,12 +3532,29 @@
         <v>8047</v>
       </c>
       <c r="U27" t="n">
-        <v>15</v>
+        <v>847.0526315789474</v>
       </c>
       <c r="V27" t="n">
-        <v>15</v>
+        <v>5167.021052631579</v>
       </c>
       <c r="W27" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X27" t="n">
+        <v>0.4636563680037474</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>5166.557396263574</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA27" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB27" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -3180,12 +3647,29 @@
         <v>8047</v>
       </c>
       <c r="U28" t="n">
+        <v>946.7058823529412</v>
+      </c>
+      <c r="V28" t="n">
+        <v>5206.882352941177</v>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X28" t="n">
+        <v>0.9136964823116547</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>5205.968656458865</v>
+      </c>
+      <c r="Z28" t="n">
         <v>10</v>
       </c>
-      <c r="V28" t="n">
+      <c r="AA28" t="n">
         <v>10</v>
       </c>
-      <c r="W28" t="inlineStr">
+      <c r="AB28" t="inlineStr">
         <is>
           <t>12/01/2026</t>
         </is>
@@ -3278,12 +3762,29 @@
         <v>8175</v>
       </c>
       <c r="U29" t="n">
+        <v>860.5263157894736</v>
+      </c>
+      <c r="V29" t="n">
+        <v>5249.210526315789</v>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X29" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>5248.7402021834</v>
+      </c>
+      <c r="Z29" t="n">
         <v>30</v>
       </c>
-      <c r="V29" t="n">
+      <c r="AA29" t="n">
         <v>30</v>
       </c>
-      <c r="W29" t="inlineStr">
+      <c r="AB29" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -3376,12 +3877,29 @@
         <v>8175</v>
       </c>
       <c r="U30" t="n">
+        <v>961.7647058823529</v>
+      </c>
+      <c r="V30" t="n">
+        <v>5289.705882352941</v>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X30" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>5288.795618514705</v>
+      </c>
+      <c r="Z30" t="n">
         <v>30</v>
       </c>
-      <c r="V30" t="n">
+      <c r="AA30" t="n">
         <v>30</v>
       </c>
-      <c r="W30" t="inlineStr">
+      <c r="AB30" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -3474,12 +3992,29 @@
         <v>7910</v>
       </c>
       <c r="U31" t="n">
-        <v>15</v>
+        <v>930.5882352941177</v>
       </c>
       <c r="V31" t="n">
-        <v>15</v>
+        <v>5118.235294117647</v>
       </c>
       <c r="W31" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X31" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>5117.32503027941</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA31" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB31" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -3572,12 +4107,29 @@
         <v>7815</v>
       </c>
       <c r="U32" t="n">
-        <v>15</v>
+        <v>947.2727272727273</v>
       </c>
       <c r="V32" t="n">
-        <v>15</v>
+        <v>5067.909090909091</v>
       </c>
       <c r="W32" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X32" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>5066.998827070855</v>
+      </c>
+      <c r="Z32" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA32" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB32" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -3670,12 +4222,29 @@
         <v>7815</v>
       </c>
       <c r="U33" t="n">
-        <v>15</v>
+        <v>928.5148514851486</v>
       </c>
       <c r="V33" t="n">
-        <v>15</v>
+        <v>5060.40594059406</v>
       </c>
       <c r="W33" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X33" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y33" t="n">
+        <v>5059.495676755823</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA33" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB33" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -3768,12 +4337,29 @@
         <v>7815</v>
       </c>
       <c r="U34" t="n">
-        <v>15</v>
+        <v>919.4117647058823</v>
       </c>
       <c r="V34" t="n">
-        <v>15</v>
+        <v>5056.764705882353</v>
       </c>
       <c r="W34" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X34" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y34" t="n">
+        <v>5055.854442044117</v>
+      </c>
+      <c r="Z34" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA34" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB34" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -3866,12 +4452,29 @@
         <v>7815</v>
       </c>
       <c r="U35" t="n">
-        <v>15</v>
+        <v>868.3333333333334</v>
       </c>
       <c r="V35" t="n">
-        <v>15</v>
+        <v>5036.333333333333</v>
       </c>
       <c r="W35" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X35" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y35" t="n">
+        <v>5035.863009200943</v>
+      </c>
+      <c r="Z35" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA35" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB35" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -3964,12 +4567,29 @@
         <v>7815</v>
       </c>
       <c r="U36" t="n">
-        <v>15</v>
+        <v>919.4117647058823</v>
       </c>
       <c r="V36" t="n">
-        <v>15</v>
+        <v>5056.764705882353</v>
       </c>
       <c r="W36" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X36" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y36" t="n">
+        <v>5055.854442044117</v>
+      </c>
+      <c r="Z36" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA36" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB36" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -4062,12 +4682,29 @@
         <v>7815</v>
       </c>
       <c r="U37" t="n">
-        <v>15</v>
+        <v>868.3333333333334</v>
       </c>
       <c r="V37" t="n">
-        <v>15</v>
+        <v>5036.333333333333</v>
       </c>
       <c r="W37" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X37" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y37" t="n">
+        <v>5035.863009200943</v>
+      </c>
+      <c r="Z37" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA37" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB37" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -4160,12 +4797,29 @@
         <v>7815</v>
       </c>
       <c r="U38" t="n">
-        <v>15</v>
+        <v>868.3333333333334</v>
       </c>
       <c r="V38" t="n">
-        <v>15</v>
+        <v>5036.333333333333</v>
       </c>
       <c r="W38" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X38" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y38" t="n">
+        <v>5035.863009200943</v>
+      </c>
+      <c r="Z38" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA38" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB38" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -4258,12 +4912,29 @@
         <v>7815</v>
       </c>
       <c r="U39" t="n">
-        <v>15</v>
+        <v>976.875</v>
       </c>
       <c r="V39" t="n">
-        <v>15</v>
+        <v>5079.75</v>
       </c>
       <c r="W39" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X39" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y39" t="n">
+        <v>5078.839736161764</v>
+      </c>
+      <c r="Z39" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA39" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB39" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -4356,12 +5027,29 @@
         <v>7790</v>
       </c>
       <c r="U40" t="n">
-        <v>15</v>
+        <v>916.4705882352941</v>
       </c>
       <c r="V40" t="n">
-        <v>15</v>
+        <v>5040.588235294118</v>
       </c>
       <c r="W40" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X40" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y40" t="n">
+        <v>5039.677971455882</v>
+      </c>
+      <c r="Z40" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA40" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB40" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -4454,12 +5142,29 @@
         <v>7773</v>
       </c>
       <c r="U41" t="n">
-        <v>15</v>
+        <v>942.1818181818181</v>
       </c>
       <c r="V41" t="n">
-        <v>15</v>
+        <v>5040.672727272728</v>
       </c>
       <c r="W41" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X41" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y41" t="n">
+        <v>5039.762463434491</v>
+      </c>
+      <c r="Z41" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA41" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB41" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -4552,12 +5257,29 @@
         <v>7773</v>
       </c>
       <c r="U42" t="n">
-        <v>15</v>
+        <v>971.625</v>
       </c>
       <c r="V42" t="n">
-        <v>15</v>
+        <v>5052.45</v>
       </c>
       <c r="W42" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X42" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y42" t="n">
+        <v>5051.539736161763</v>
+      </c>
+      <c r="Z42" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA42" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB42" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -4650,12 +5372,29 @@
         <v>7773</v>
       </c>
       <c r="U43" t="n">
-        <v>15</v>
+        <v>961.6082474226804</v>
       </c>
       <c r="V43" t="n">
-        <v>15</v>
+        <v>5048.443298969072</v>
       </c>
       <c r="W43" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X43" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y43" t="n">
+        <v>5047.533035130836</v>
+      </c>
+      <c r="Z43" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA43" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB43" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -4748,12 +5487,29 @@
         <v>7773</v>
       </c>
       <c r="U44" t="n">
+        <v>961.6082474226804</v>
+      </c>
+      <c r="V44" t="n">
+        <v>5048.443298969072</v>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X44" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y44" t="n">
+        <v>5047.533035130836</v>
+      </c>
+      <c r="Z44" t="n">
         <v>6</v>
       </c>
-      <c r="V44" t="n">
+      <c r="AA44" t="n">
         <v>6</v>
       </c>
-      <c r="W44" t="inlineStr">
+      <c r="AB44" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -4846,12 +5602,29 @@
         <v>7773</v>
       </c>
       <c r="U45" t="n">
-        <v>15</v>
+        <v>914.4705882352941</v>
       </c>
       <c r="V45" t="n">
-        <v>15</v>
+        <v>5029.588235294118</v>
       </c>
       <c r="W45" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X45" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y45" t="n">
+        <v>5028.677971455882</v>
+      </c>
+      <c r="Z45" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA45" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB45" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -4944,12 +5717,29 @@
         <v>7773</v>
       </c>
       <c r="U46" t="n">
-        <v>15</v>
+        <v>863.6666666666666</v>
       </c>
       <c r="V46" t="n">
-        <v>15</v>
+        <v>5009.266666666666</v>
       </c>
       <c r="W46" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X46" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y46" t="n">
+        <v>5008.796342534277</v>
+      </c>
+      <c r="Z46" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA46" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB46" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -5042,12 +5832,29 @@
         <v>7773</v>
       </c>
       <c r="U47" t="n">
-        <v>15</v>
+        <v>942.1818181818181</v>
       </c>
       <c r="V47" t="n">
-        <v>15</v>
+        <v>5040.672727272728</v>
       </c>
       <c r="W47" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X47" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y47" t="n">
+        <v>5039.762463434491</v>
+      </c>
+      <c r="Z47" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA47" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB47" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -5140,12 +5947,29 @@
         <v>7773</v>
       </c>
       <c r="U48" t="n">
-        <v>15</v>
+        <v>863.6666666666666</v>
       </c>
       <c r="V48" t="n">
-        <v>15</v>
+        <v>5009.266666666666</v>
       </c>
       <c r="W48" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X48" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y48" t="n">
+        <v>5008.796342534277</v>
+      </c>
+      <c r="Z48" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA48" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB48" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -5238,12 +6062,29 @@
         <v>7718</v>
       </c>
       <c r="U49" t="n">
-        <v>15</v>
+        <v>857.5555555555555</v>
       </c>
       <c r="V49" t="n">
-        <v>15</v>
+        <v>4973.822222222222</v>
       </c>
       <c r="W49" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X49" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y49" t="n">
+        <v>4973.351898089833</v>
+      </c>
+      <c r="Z49" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA49" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB49" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -5336,12 +6177,29 @@
         <v>7617</v>
       </c>
       <c r="U50" t="n">
-        <v>15</v>
+        <v>952.125</v>
       </c>
       <c r="V50" t="n">
-        <v>15</v>
+        <v>4951.05</v>
       </c>
       <c r="W50" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X50" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y50" t="n">
+        <v>4950.139736161764</v>
+      </c>
+      <c r="Z50" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA50" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB50" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -5434,12 +6292,29 @@
         <v>7617</v>
       </c>
       <c r="U51" t="n">
-        <v>15</v>
+        <v>896.1176470588235</v>
       </c>
       <c r="V51" t="n">
-        <v>15</v>
+        <v>4928.64705882353</v>
       </c>
       <c r="W51" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X51" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y51" t="n">
+        <v>4927.736794985293</v>
+      </c>
+      <c r="Z51" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA51" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB51" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -5532,12 +6407,29 @@
         <v>7617</v>
       </c>
       <c r="U52" t="n">
+        <v>896.1176470588235</v>
+      </c>
+      <c r="V52" t="n">
+        <v>4928.64705882353</v>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X52" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y52" t="n">
+        <v>4927.736794985293</v>
+      </c>
+      <c r="Z52" t="n">
         <v>5</v>
       </c>
-      <c r="V52" t="n">
+      <c r="AA52" t="n">
         <v>5</v>
       </c>
-      <c r="W52" t="inlineStr">
+      <c r="AB52" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -5630,12 +6522,29 @@
         <v>7617</v>
       </c>
       <c r="U53" t="n">
-        <v>15</v>
+        <v>801.7894736842105</v>
       </c>
       <c r="V53" t="n">
-        <v>15</v>
+        <v>4890.915789473684</v>
       </c>
       <c r="W53" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X53" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y53" t="n">
+        <v>4890.445465341294</v>
+      </c>
+      <c r="Z53" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA53" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB53" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -5728,12 +6637,29 @@
         <v>7617</v>
       </c>
       <c r="U54" t="n">
-        <v>15</v>
+        <v>896.1176470588235</v>
       </c>
       <c r="V54" t="n">
-        <v>15</v>
+        <v>4928.64705882353</v>
       </c>
       <c r="W54" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X54" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y54" t="n">
+        <v>4927.736794985293</v>
+      </c>
+      <c r="Z54" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA54" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB54" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -5826,12 +6752,29 @@
         <v>7617</v>
       </c>
       <c r="U55" t="n">
-        <v>15</v>
+        <v>896.1176470588235</v>
       </c>
       <c r="V55" t="n">
-        <v>15</v>
+        <v>4928.64705882353</v>
       </c>
       <c r="W55" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X55" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y55" t="n">
+        <v>4927.736794985293</v>
+      </c>
+      <c r="Z55" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA55" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB55" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -5924,12 +6867,29 @@
         <v>7374</v>
       </c>
       <c r="U56" t="n">
+        <v>776.2105263157895</v>
+      </c>
+      <c r="V56" t="n">
+        <v>4734.884210526316</v>
+      </c>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X56" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y56" t="n">
+        <v>4734.413886393926</v>
+      </c>
+      <c r="Z56" t="n">
         <v>2</v>
       </c>
-      <c r="V56" t="n">
+      <c r="AA56" t="n">
         <v>2</v>
       </c>
-      <c r="W56" t="inlineStr">
+      <c r="AB56" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
@@ -6022,12 +6982,29 @@
         <v>7364</v>
       </c>
       <c r="U57" t="n">
+        <v>775.1578947368421</v>
+      </c>
+      <c r="V57" t="n">
+        <v>4728.463157894736</v>
+      </c>
+      <c r="W57" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X57" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y57" t="n">
+        <v>4727.992833762347</v>
+      </c>
+      <c r="Z57" t="n">
         <v>30</v>
       </c>
-      <c r="V57" t="n">
+      <c r="AA57" t="n">
         <v>30</v>
       </c>
-      <c r="W57" t="inlineStr">
+      <c r="AB57" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -6120,12 +7097,29 @@
         <v>7364</v>
       </c>
       <c r="U58" t="n">
+        <v>866.3529411764706</v>
+      </c>
+      <c r="V58" t="n">
+        <v>4764.941176470588</v>
+      </c>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X58" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y58" t="n">
+        <v>4764.030912632352</v>
+      </c>
+      <c r="Z58" t="n">
         <v>30</v>
       </c>
-      <c r="V58" t="n">
+      <c r="AA58" t="n">
         <v>30</v>
       </c>
-      <c r="W58" t="inlineStr">
+      <c r="AB58" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -6218,12 +7212,29 @@
         <v>7140</v>
       </c>
       <c r="U59" t="n">
-        <v>15</v>
+        <v>840</v>
       </c>
       <c r="V59" t="n">
-        <v>15</v>
+        <v>4620</v>
       </c>
       <c r="W59" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X59" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y59" t="n">
+        <v>4619.089736161764</v>
+      </c>
+      <c r="Z59" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA59" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB59" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -6316,12 +7327,29 @@
         <v>7045</v>
       </c>
       <c r="U60" t="n">
-        <v>15</v>
+        <v>853.939393939394</v>
       </c>
       <c r="V60" t="n">
-        <v>15</v>
+        <v>4568.575757575758</v>
       </c>
       <c r="W60" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X60" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y60" t="n">
+        <v>4567.665493737522</v>
+      </c>
+      <c r="Z60" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA60" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB60" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -6414,12 +7442,29 @@
         <v>7045</v>
       </c>
       <c r="U61" t="n">
-        <v>15</v>
+        <v>828.8235294117648</v>
       </c>
       <c r="V61" t="n">
-        <v>15</v>
+        <v>4558.529411764706</v>
       </c>
       <c r="W61" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X61" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y61" t="n">
+        <v>4557.61914792647</v>
+      </c>
+      <c r="Z61" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA61" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB61" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -6512,12 +7557,29 @@
         <v>7045</v>
       </c>
       <c r="U62" t="n">
-        <v>15</v>
+        <v>782.7777777777778</v>
       </c>
       <c r="V62" t="n">
-        <v>15</v>
+        <v>4540.111111111111</v>
       </c>
       <c r="W62" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X62" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y62" t="n">
+        <v>4539.640786978722</v>
+      </c>
+      <c r="Z62" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA62" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB62" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -6610,12 +7672,29 @@
         <v>7045</v>
       </c>
       <c r="U63" t="n">
-        <v>15</v>
+        <v>837.0297029702971</v>
       </c>
       <c r="V63" t="n">
-        <v>15</v>
+        <v>4561.811881188119</v>
       </c>
       <c r="W63" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X63" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y63" t="n">
+        <v>4560.901617349882</v>
+      </c>
+      <c r="Z63" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA63" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB63" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -6708,12 +7787,29 @@
         <v>7045</v>
       </c>
       <c r="U64" t="n">
-        <v>15</v>
+        <v>880.625</v>
       </c>
       <c r="V64" t="n">
-        <v>15</v>
+        <v>4579.25</v>
       </c>
       <c r="W64" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X64" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y64" t="n">
+        <v>4578.339736161764</v>
+      </c>
+      <c r="Z64" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA64" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB64" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -6806,12 +7902,29 @@
         <v>7045</v>
       </c>
       <c r="U65" t="n">
-        <v>15</v>
+        <v>782.7777777777778</v>
       </c>
       <c r="V65" t="n">
-        <v>15</v>
+        <v>4540.111111111111</v>
       </c>
       <c r="W65" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X65" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y65" t="n">
+        <v>4539.640786978722</v>
+      </c>
+      <c r="Z65" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA65" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB65" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -6904,12 +8017,29 @@
         <v>7045</v>
       </c>
       <c r="U66" t="n">
+        <v>782.7777777777778</v>
+      </c>
+      <c r="V66" t="n">
+        <v>4540.111111111111</v>
+      </c>
+      <c r="W66" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X66" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y66" t="n">
+        <v>4539.640786978722</v>
+      </c>
+      <c r="Z66" t="n">
         <v>6</v>
       </c>
-      <c r="V66" t="n">
+      <c r="AA66" t="n">
         <v>6</v>
       </c>
-      <c r="W66" t="inlineStr">
+      <c r="AB66" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -7002,12 +8132,29 @@
         <v>7005</v>
       </c>
       <c r="U67" t="n">
-        <v>15</v>
+        <v>849.0909090909091</v>
       </c>
       <c r="V67" t="n">
-        <v>15</v>
+        <v>4542.636363636364</v>
       </c>
       <c r="W67" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X67" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y67" t="n">
+        <v>4541.726099798128</v>
+      </c>
+      <c r="Z67" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA67" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB67" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -7100,12 +8247,29 @@
         <v>7005</v>
       </c>
       <c r="U68" t="n">
-        <v>15</v>
+        <v>849.0909090909091</v>
       </c>
       <c r="V68" t="n">
-        <v>15</v>
+        <v>4542.636363636364</v>
       </c>
       <c r="W68" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X68" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y68" t="n">
+        <v>4541.726099798128</v>
+      </c>
+      <c r="Z68" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA68" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB68" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -7198,12 +8362,29 @@
         <v>7005</v>
       </c>
       <c r="U69" t="n">
-        <v>15</v>
+        <v>866.5979381443299</v>
       </c>
       <c r="V69" t="n">
-        <v>15</v>
+        <v>4549.639175257732</v>
       </c>
       <c r="W69" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X69" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y69" t="n">
+        <v>4548.728911419495</v>
+      </c>
+      <c r="Z69" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA69" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB69" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -7296,12 +8477,29 @@
         <v>7005</v>
       </c>
       <c r="U70" t="n">
-        <v>15</v>
+        <v>778.3333333333334</v>
       </c>
       <c r="V70" t="n">
-        <v>15</v>
+        <v>4514.333333333333</v>
       </c>
       <c r="W70" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X70" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y70" t="n">
+        <v>4513.863009200943</v>
+      </c>
+      <c r="Z70" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA70" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB70" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -7394,12 +8592,29 @@
         <v>7005</v>
       </c>
       <c r="U71" t="n">
-        <v>15</v>
+        <v>866.5979381443299</v>
       </c>
       <c r="V71" t="n">
-        <v>15</v>
+        <v>4549.639175257732</v>
       </c>
       <c r="W71" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X71" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y71" t="n">
+        <v>4548.728911419495</v>
+      </c>
+      <c r="Z71" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA71" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB71" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -7492,12 +8707,29 @@
         <v>7005</v>
       </c>
       <c r="U72" t="n">
-        <v>15</v>
+        <v>778.3333333333334</v>
       </c>
       <c r="V72" t="n">
-        <v>15</v>
+        <v>4514.333333333333</v>
       </c>
       <c r="W72" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X72" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y72" t="n">
+        <v>4513.863009200943</v>
+      </c>
+      <c r="Z72" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA72" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB72" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -7590,12 +8822,29 @@
         <v>6953</v>
       </c>
       <c r="U73" t="n">
-        <v>15</v>
+        <v>772.5555555555555</v>
       </c>
       <c r="V73" t="n">
-        <v>15</v>
+        <v>4480.822222222222</v>
       </c>
       <c r="W73" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X73" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y73" t="n">
+        <v>4480.351898089833</v>
+      </c>
+      <c r="Z73" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA73" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB73" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -7688,12 +8937,29 @@
         <v>6880</v>
       </c>
       <c r="U74" t="n">
-        <v>15</v>
+        <v>809.4117647058823</v>
       </c>
       <c r="V74" t="n">
-        <v>15</v>
+        <v>4451.764705882353</v>
       </c>
       <c r="W74" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X74" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y74" t="n">
+        <v>4450.854442044117</v>
+      </c>
+      <c r="Z74" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA74" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB74" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -7786,12 +9052,29 @@
         <v>6880</v>
       </c>
       <c r="U75" t="n">
-        <v>15</v>
+        <v>809.4117647058823</v>
       </c>
       <c r="V75" t="n">
-        <v>15</v>
+        <v>4451.764705882353</v>
       </c>
       <c r="W75" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X75" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y75" t="n">
+        <v>4450.854442044117</v>
+      </c>
+      <c r="Z75" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA75" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB75" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -7884,12 +9167,29 @@
         <v>6880</v>
       </c>
       <c r="U76" t="n">
+        <v>724.2105263157895</v>
+      </c>
+      <c r="V76" t="n">
+        <v>4417.684210526316</v>
+      </c>
+      <c r="W76" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X76" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y76" t="n">
+        <v>4417.213886393926</v>
+      </c>
+      <c r="Z76" t="n">
         <v>14</v>
       </c>
-      <c r="V76" t="n">
+      <c r="AA76" t="n">
         <v>14</v>
       </c>
-      <c r="W76" t="inlineStr">
+      <c r="AB76" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -7982,12 +9282,29 @@
         <v>6880</v>
       </c>
       <c r="U77" t="n">
-        <v>15</v>
+        <v>809.4117647058823</v>
       </c>
       <c r="V77" t="n">
-        <v>15</v>
+        <v>4451.764705882353</v>
       </c>
       <c r="W77" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X77" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y77" t="n">
+        <v>4450.854442044117</v>
+      </c>
+      <c r="Z77" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA77" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB77" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -8080,12 +9397,29 @@
         <v>6880</v>
       </c>
       <c r="U78" t="n">
-        <v>15</v>
+        <v>860</v>
       </c>
       <c r="V78" t="n">
-        <v>15</v>
+        <v>4472</v>
       </c>
       <c r="W78" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X78" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y78" t="n">
+        <v>4471.089736161764</v>
+      </c>
+      <c r="Z78" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA78" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB78" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -8178,12 +9512,29 @@
         <v>6624</v>
       </c>
       <c r="U79" t="n">
-        <v>15</v>
+        <v>779.2941176470588</v>
       </c>
       <c r="V79" t="n">
-        <v>15</v>
+        <v>4286.117647058823</v>
       </c>
       <c r="W79" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X79" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y79" t="n">
+        <v>4285.207383220587</v>
+      </c>
+      <c r="Z79" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA79" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB79" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -8276,12 +9627,29 @@
         <v>6562</v>
       </c>
       <c r="U80" t="n">
+        <v>772</v>
+      </c>
+      <c r="V80" t="n">
+        <v>4246</v>
+      </c>
+      <c r="W80" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X80" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y80" t="n">
+        <v>4245.089736161764</v>
+      </c>
+      <c r="Z80" t="n">
         <v>7</v>
       </c>
-      <c r="V80" t="n">
+      <c r="AA80" t="n">
         <v>7</v>
       </c>
-      <c r="W80" t="inlineStr">
+      <c r="AB80" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -8374,12 +9742,29 @@
         <v>6248</v>
       </c>
       <c r="U81" t="n">
+        <v>735.0588235294117</v>
+      </c>
+      <c r="V81" t="n">
+        <v>4042.823529411764</v>
+      </c>
+      <c r="W81" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X81" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y81" t="n">
+        <v>4041.913265573528</v>
+      </c>
+      <c r="Z81" t="n">
         <v>6</v>
       </c>
-      <c r="V81" t="n">
+      <c r="AA81" t="n">
         <v>6</v>
       </c>
-      <c r="W81" t="inlineStr">
+      <c r="AB81" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -8472,12 +9857,29 @@
         <v>6238</v>
       </c>
       <c r="U82" t="n">
+        <v>779.75</v>
+      </c>
+      <c r="V82" t="n">
+        <v>4054.7</v>
+      </c>
+      <c r="W82" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X82" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y82" t="n">
+        <v>4053.789736161763</v>
+      </c>
+      <c r="Z82" t="n">
         <v>7</v>
       </c>
-      <c r="V82" t="n">
+      <c r="AA82" t="n">
         <v>7</v>
       </c>
-      <c r="W82" t="inlineStr">
+      <c r="AB82" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -8570,12 +9972,29 @@
         <v>6231</v>
       </c>
       <c r="U83" t="n">
+        <v>778.875</v>
+      </c>
+      <c r="V83" t="n">
+        <v>4050.15</v>
+      </c>
+      <c r="W83" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X83" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y83" t="n">
+        <v>4049.239736161764</v>
+      </c>
+      <c r="Z83" t="n">
         <v>9</v>
       </c>
-      <c r="V83" t="n">
+      <c r="AA83" t="n">
         <v>9</v>
       </c>
-      <c r="W83" t="inlineStr">
+      <c r="AB83" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -8668,12 +10087,29 @@
         <v>6025</v>
       </c>
       <c r="U84" t="n">
+        <v>753.125</v>
+      </c>
+      <c r="V84" t="n">
+        <v>3916.25</v>
+      </c>
+      <c r="W84" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X84" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y84" t="n">
+        <v>3915.339736161764</v>
+      </c>
+      <c r="Z84" t="n">
         <v>4</v>
       </c>
-      <c r="V84" t="n">
+      <c r="AA84" t="n">
         <v>4</v>
       </c>
-      <c r="W84" t="inlineStr">
+      <c r="AB84" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -8766,12 +10202,29 @@
         <v>5882</v>
       </c>
       <c r="U85" t="n">
+        <v>692</v>
+      </c>
+      <c r="V85" t="n">
+        <v>3806</v>
+      </c>
+      <c r="W85" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X85" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y85" t="n">
+        <v>3805.089736161764</v>
+      </c>
+      <c r="Z85" t="n">
         <v>11</v>
       </c>
-      <c r="V85" t="n">
+      <c r="AA85" t="n">
         <v>11</v>
       </c>
-      <c r="W85" t="inlineStr">
+      <c r="AB85" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -8864,12 +10317,29 @@
         <v>5664</v>
       </c>
       <c r="U86" t="n">
+        <v>666.3529411764706</v>
+      </c>
+      <c r="V86" t="n">
+        <v>3664.941176470588</v>
+      </c>
+      <c r="W86" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X86" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y86" t="n">
+        <v>3664.030912632352</v>
+      </c>
+      <c r="Z86" t="n">
         <v>2</v>
       </c>
-      <c r="V86" t="n">
+      <c r="AA86" t="n">
         <v>2</v>
       </c>
-      <c r="W86" t="inlineStr">
+      <c r="AB86" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -8962,12 +10432,29 @@
         <v>8153</v>
       </c>
       <c r="U87" t="n">
+        <v>959.1764705882352</v>
+      </c>
+      <c r="V87" t="n">
+        <v>5275.470588235295</v>
+      </c>
+      <c r="W87" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X87" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y87" t="n">
+        <v>5274.560324397058</v>
+      </c>
+      <c r="Z87" t="n">
         <v>30</v>
       </c>
-      <c r="V87" t="n">
+      <c r="AA87" t="n">
         <v>30</v>
       </c>
-      <c r="W87" t="inlineStr">
+      <c r="AB87" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -9060,12 +10547,29 @@
         <v>8153</v>
       </c>
       <c r="U88" t="n">
+        <v>858.2105263157895</v>
+      </c>
+      <c r="V88" t="n">
+        <v>5235.084210526316</v>
+      </c>
+      <c r="W88" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X88" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y88" t="n">
+        <v>5234.613886393927</v>
+      </c>
+      <c r="Z88" t="n">
         <v>30</v>
       </c>
-      <c r="V88" t="n">
+      <c r="AA88" t="n">
         <v>30</v>
       </c>
-      <c r="W88" t="inlineStr">
+      <c r="AB88" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -9158,12 +10662,29 @@
         <v>7882</v>
       </c>
       <c r="U89" t="n">
+        <v>927.2941176470588</v>
+      </c>
+      <c r="V89" t="n">
+        <v>5100.117647058823</v>
+      </c>
+      <c r="W89" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X89" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y89" t="n">
+        <v>5099.207383220587</v>
+      </c>
+      <c r="Z89" t="n">
         <v>17</v>
       </c>
-      <c r="V89" t="n">
+      <c r="AA89" t="n">
         <v>17</v>
       </c>
-      <c r="W89" t="inlineStr">
+      <c r="AB89" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -9256,12 +10777,29 @@
         <v>7791</v>
       </c>
       <c r="U90" t="n">
-        <v>15</v>
+        <v>944.3636363636364</v>
       </c>
       <c r="V90" t="n">
-        <v>15</v>
+        <v>5052.345454545454</v>
       </c>
       <c r="W90" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X90" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y90" t="n">
+        <v>5051.435190707218</v>
+      </c>
+      <c r="Z90" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA90" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB90" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -9354,12 +10892,29 @@
         <v>7791</v>
       </c>
       <c r="U91" t="n">
-        <v>15</v>
+        <v>916.5882352941177</v>
       </c>
       <c r="V91" t="n">
-        <v>15</v>
+        <v>5041.235294117647</v>
       </c>
       <c r="W91" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X91" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y91" t="n">
+        <v>5040.32503027941</v>
+      </c>
+      <c r="Z91" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA91" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB91" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -9452,12 +11007,29 @@
         <v>7791</v>
       </c>
       <c r="U92" t="n">
-        <v>15</v>
+        <v>916.5882352941177</v>
       </c>
       <c r="V92" t="n">
-        <v>15</v>
+        <v>5041.235294117647</v>
       </c>
       <c r="W92" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X92" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y92" t="n">
+        <v>5040.32503027941</v>
+      </c>
+      <c r="Z92" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA92" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB92" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -9550,12 +11122,29 @@
         <v>7791</v>
       </c>
       <c r="U93" t="n">
-        <v>15</v>
+        <v>865.6666666666666</v>
       </c>
       <c r="V93" t="n">
-        <v>15</v>
+        <v>5020.866666666666</v>
       </c>
       <c r="W93" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X93" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y93" t="n">
+        <v>5020.396342534276</v>
+      </c>
+      <c r="Z93" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA93" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB93" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -9648,12 +11237,29 @@
         <v>7791</v>
       </c>
       <c r="U94" t="n">
-        <v>15</v>
+        <v>973.875</v>
       </c>
       <c r="V94" t="n">
-        <v>15</v>
+        <v>5064.15</v>
       </c>
       <c r="W94" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X94" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y94" t="n">
+        <v>5063.239736161763</v>
+      </c>
+      <c r="Z94" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA94" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB94" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -9746,12 +11352,29 @@
         <v>7791</v>
       </c>
       <c r="U95" t="n">
-        <v>15</v>
+        <v>865.6666666666666</v>
       </c>
       <c r="V95" t="n">
-        <v>15</v>
+        <v>5020.866666666666</v>
       </c>
       <c r="W95" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X95" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y95" t="n">
+        <v>5020.396342534276</v>
+      </c>
+      <c r="Z95" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA95" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB95" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -9844,12 +11467,29 @@
         <v>7791</v>
       </c>
       <c r="U96" t="n">
-        <v>15</v>
+        <v>865.6666666666666</v>
       </c>
       <c r="V96" t="n">
-        <v>15</v>
+        <v>5020.866666666666</v>
       </c>
       <c r="W96" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X96" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y96" t="n">
+        <v>5020.396342534276</v>
+      </c>
+      <c r="Z96" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA96" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB96" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -9942,12 +11582,29 @@
         <v>7791</v>
       </c>
       <c r="U97" t="n">
-        <v>15</v>
+        <v>925.6633663366338</v>
       </c>
       <c r="V97" t="n">
-        <v>15</v>
+        <v>5044.865346534653</v>
       </c>
       <c r="W97" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X97" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y97" t="n">
+        <v>5043.955082696417</v>
+      </c>
+      <c r="Z97" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA97" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB97" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -10040,12 +11697,29 @@
         <v>7773</v>
       </c>
       <c r="U98" t="n">
+        <v>818.2105263157895</v>
+      </c>
+      <c r="V98" t="n">
+        <v>4991.084210526316</v>
+      </c>
+      <c r="W98" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X98" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y98" t="n">
+        <v>4990.613886393927</v>
+      </c>
+      <c r="Z98" t="n">
         <v>10</v>
       </c>
-      <c r="V98" t="n">
+      <c r="AA98" t="n">
         <v>10</v>
       </c>
-      <c r="W98" t="inlineStr">
+      <c r="AB98" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -10138,12 +11812,29 @@
         <v>7763</v>
       </c>
       <c r="U99" t="n">
+        <v>913.2941176470588</v>
+      </c>
+      <c r="V99" t="n">
+        <v>5023.117647058823</v>
+      </c>
+      <c r="W99" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X99" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y99" t="n">
+        <v>5022.207383220587</v>
+      </c>
+      <c r="Z99" t="n">
         <v>17</v>
       </c>
-      <c r="V99" t="n">
+      <c r="AA99" t="n">
         <v>17</v>
       </c>
-      <c r="W99" t="inlineStr">
+      <c r="AB99" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -10236,12 +11927,29 @@
         <v>7763</v>
       </c>
       <c r="U100" t="n">
-        <v>15</v>
+        <v>862.5555555555555</v>
       </c>
       <c r="V100" t="n">
-        <v>15</v>
+        <v>5002.822222222222</v>
       </c>
       <c r="W100" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X100" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y100" t="n">
+        <v>5002.351898089833</v>
+      </c>
+      <c r="Z100" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA100" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB100" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -10334,12 +12042,29 @@
         <v>7763</v>
       </c>
       <c r="U101" t="n">
-        <v>15</v>
+        <v>960.3711340206185</v>
       </c>
       <c r="V101" t="n">
-        <v>15</v>
+        <v>5041.948453608247</v>
       </c>
       <c r="W101" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X101" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y101" t="n">
+        <v>5041.038189770011</v>
+      </c>
+      <c r="Z101" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA101" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB101" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -10432,12 +12157,29 @@
         <v>7763</v>
       </c>
       <c r="U102" t="n">
-        <v>15</v>
+        <v>960.3711340206185</v>
       </c>
       <c r="V102" t="n">
-        <v>15</v>
+        <v>5041.948453608247</v>
       </c>
       <c r="W102" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X102" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y102" t="n">
+        <v>5041.038189770011</v>
+      </c>
+      <c r="Z102" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA102" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB102" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -10530,12 +12272,29 @@
         <v>7763</v>
       </c>
       <c r="U103" t="n">
-        <v>15</v>
+        <v>940.969696969697</v>
       </c>
       <c r="V103" t="n">
-        <v>15</v>
+        <v>5034.187878787879</v>
       </c>
       <c r="W103" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X103" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y103" t="n">
+        <v>5033.277614949642</v>
+      </c>
+      <c r="Z103" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA103" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB103" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -10628,12 +12387,29 @@
         <v>7763</v>
       </c>
       <c r="U104" t="n">
-        <v>15</v>
+        <v>940.969696969697</v>
       </c>
       <c r="V104" t="n">
-        <v>15</v>
+        <v>5034.187878787879</v>
       </c>
       <c r="W104" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X104" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y104" t="n">
+        <v>5033.277614949642</v>
+      </c>
+      <c r="Z104" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA104" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB104" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -10726,12 +12502,29 @@
         <v>7763</v>
       </c>
       <c r="U105" t="n">
-        <v>15</v>
+        <v>862.5555555555555</v>
       </c>
       <c r="V105" t="n">
-        <v>15</v>
+        <v>5002.822222222222</v>
       </c>
       <c r="W105" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X105" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y105" t="n">
+        <v>5002.351898089833</v>
+      </c>
+      <c r="Z105" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA105" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB105" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -10824,12 +12617,29 @@
         <v>7763</v>
       </c>
       <c r="U106" t="n">
-        <v>15</v>
+        <v>970.375</v>
       </c>
       <c r="V106" t="n">
-        <v>15</v>
+        <v>5045.95</v>
       </c>
       <c r="W106" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X106" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y106" t="n">
+        <v>5045.039736161763</v>
+      </c>
+      <c r="Z106" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA106" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB106" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -10922,12 +12732,29 @@
         <v>7699</v>
       </c>
       <c r="U107" t="n">
-        <v>15</v>
+        <v>855.4444444444445</v>
       </c>
       <c r="V107" t="n">
-        <v>15</v>
+        <v>4961.577777777778</v>
       </c>
       <c r="W107" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X107" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y107" t="n">
+        <v>4961.107453645388</v>
+      </c>
+      <c r="Z107" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA107" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB107" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -11020,12 +12847,29 @@
         <v>7580</v>
       </c>
       <c r="U108" t="n">
-        <v>15</v>
+        <v>891.7647058823529</v>
       </c>
       <c r="V108" t="n">
-        <v>15</v>
+        <v>4904.705882352941</v>
       </c>
       <c r="W108" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X108" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y108" t="n">
+        <v>4903.795618514705</v>
+      </c>
+      <c r="Z108" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA108" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB108" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -11118,12 +12962,29 @@
         <v>7580</v>
       </c>
       <c r="U109" t="n">
-        <v>15</v>
+        <v>891.7647058823529</v>
       </c>
       <c r="V109" t="n">
-        <v>15</v>
+        <v>4904.705882352941</v>
       </c>
       <c r="W109" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X109" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y109" t="n">
+        <v>4903.795618514705</v>
+      </c>
+      <c r="Z109" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA109" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB109" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -11216,12 +13077,29 @@
         <v>7580</v>
       </c>
       <c r="U110" t="n">
+        <v>947.5</v>
+      </c>
+      <c r="V110" t="n">
+        <v>4927</v>
+      </c>
+      <c r="W110" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X110" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y110" t="n">
+        <v>4926.089736161764</v>
+      </c>
+      <c r="Z110" t="n">
         <v>14</v>
       </c>
-      <c r="V110" t="n">
+      <c r="AA110" t="n">
         <v>14</v>
       </c>
-      <c r="W110" t="inlineStr">
+      <c r="AB110" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -11314,12 +13192,29 @@
         <v>7580</v>
       </c>
       <c r="U111" t="n">
-        <v>15</v>
+        <v>891.7647058823529</v>
       </c>
       <c r="V111" t="n">
-        <v>15</v>
+        <v>4904.705882352941</v>
       </c>
       <c r="W111" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X111" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y111" t="n">
+        <v>4903.795618514705</v>
+      </c>
+      <c r="Z111" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA111" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB111" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -11412,12 +13307,29 @@
         <v>7580</v>
       </c>
       <c r="U112" t="n">
-        <v>15</v>
+        <v>891.7647058823529</v>
       </c>
       <c r="V112" t="n">
-        <v>15</v>
+        <v>4904.705882352941</v>
       </c>
       <c r="W112" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X112" t="n">
+        <v>0.9102638382366166</v>
+      </c>
+      <c r="Y112" t="n">
+        <v>4903.795618514705</v>
+      </c>
+      <c r="Z112" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA112" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB112" t="inlineStr">
         <is>
           <t>15/01/2026</t>
         </is>
@@ -11510,12 +13422,29 @@
         <v>8212</v>
       </c>
       <c r="U113" t="n">
+        <v>864.421052631579</v>
+      </c>
+      <c r="V113" t="n">
+        <v>5272.968421052631</v>
+      </c>
+      <c r="W113" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X113" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y113" t="n">
+        <v>5272.498096920242</v>
+      </c>
+      <c r="Z113" t="n">
         <v>30</v>
       </c>
-      <c r="V113" t="n">
+      <c r="AA113" t="n">
         <v>30</v>
       </c>
-      <c r="W113" t="inlineStr">
+      <c r="AB113" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -11608,12 +13537,29 @@
         <v>8212</v>
       </c>
       <c r="U114" t="n">
+        <v>966.1176470588235</v>
+      </c>
+      <c r="V114" t="n">
+        <v>5313.64705882353</v>
+      </c>
+      <c r="W114" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X114" t="n">
+        <v>0.9099162135155621</v>
+      </c>
+      <c r="Y114" t="n">
+        <v>5312.737142610014</v>
+      </c>
+      <c r="Z114" t="n">
         <v>30</v>
       </c>
-      <c r="V114" t="n">
+      <c r="AA114" t="n">
         <v>30</v>
       </c>
-      <c r="W114" t="inlineStr">
+      <c r="AB114" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -11706,12 +13652,29 @@
         <v>8008</v>
       </c>
       <c r="U115" t="n">
+        <v>842.9473684210526</v>
+      </c>
+      <c r="V115" t="n">
+        <v>5141.978947368421</v>
+      </c>
+      <c r="W115" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X115" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y115" t="n">
+        <v>5141.508623236032</v>
+      </c>
+      <c r="Z115" t="n">
         <v>12</v>
       </c>
-      <c r="V115" t="n">
+      <c r="AA115" t="n">
         <v>12</v>
       </c>
-      <c r="W115" t="inlineStr">
+      <c r="AB115" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -11804,12 +13767,29 @@
         <v>7996</v>
       </c>
       <c r="U116" t="n">
-        <v>15</v>
+        <v>888.4444444444445</v>
       </c>
       <c r="V116" t="n">
-        <v>15</v>
+        <v>5152.977777777777</v>
       </c>
       <c r="W116" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X116" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y116" t="n">
+        <v>5152.507453645388</v>
+      </c>
+      <c r="Z116" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA116" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB116" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -11902,12 +13882,29 @@
         <v>7996</v>
       </c>
       <c r="U117" t="n">
+        <v>999.5</v>
+      </c>
+      <c r="V117" t="n">
+        <v>5197.4</v>
+      </c>
+      <c r="W117" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X117" t="n">
+        <v>0.9099162135155621</v>
+      </c>
+      <c r="Y117" t="n">
+        <v>5196.490083786484</v>
+      </c>
+      <c r="Z117" t="n">
         <v>30</v>
       </c>
-      <c r="V117" t="n">
+      <c r="AA117" t="n">
         <v>30</v>
       </c>
-      <c r="W117" t="inlineStr">
+      <c r="AB117" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -12000,12 +13997,29 @@
         <v>7996</v>
       </c>
       <c r="U118" t="n">
+        <v>940.7058823529412</v>
+      </c>
+      <c r="V118" t="n">
+        <v>5173.882352941176</v>
+      </c>
+      <c r="W118" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X118" t="n">
+        <v>0.9099162135155621</v>
+      </c>
+      <c r="Y118" t="n">
+        <v>5172.97243672766</v>
+      </c>
+      <c r="Z118" t="n">
         <v>30</v>
       </c>
-      <c r="V118" t="n">
+      <c r="AA118" t="n">
         <v>30</v>
       </c>
-      <c r="W118" t="inlineStr">
+      <c r="AB118" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -12098,12 +14112,29 @@
         <v>7996</v>
       </c>
       <c r="U119" t="n">
-        <v>15</v>
+        <v>969.2121212121212</v>
       </c>
       <c r="V119" t="n">
-        <v>15</v>
+        <v>5185.284848484848</v>
       </c>
       <c r="W119" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X119" t="n">
+        <v>0.9099162135155621</v>
+      </c>
+      <c r="Y119" t="n">
+        <v>5184.374932271333</v>
+      </c>
+      <c r="Z119" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA119" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB119" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -12196,12 +14227,29 @@
         <v>7996</v>
       </c>
       <c r="U120" t="n">
+        <v>989.1958762886597</v>
+      </c>
+      <c r="V120" t="n">
+        <v>5193.278350515463</v>
+      </c>
+      <c r="W120" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X120" t="n">
+        <v>0.9099162135155621</v>
+      </c>
+      <c r="Y120" t="n">
+        <v>5192.368434301948</v>
+      </c>
+      <c r="Z120" t="n">
         <v>30</v>
       </c>
-      <c r="V120" t="n">
+      <c r="AA120" t="n">
         <v>30</v>
       </c>
-      <c r="W120" t="inlineStr">
+      <c r="AB120" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -12294,12 +14342,29 @@
         <v>7996</v>
       </c>
       <c r="U121" t="n">
+        <v>989.1958762886597</v>
+      </c>
+      <c r="V121" t="n">
+        <v>5193.278350515463</v>
+      </c>
+      <c r="W121" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X121" t="n">
+        <v>0.9099162135155621</v>
+      </c>
+      <c r="Y121" t="n">
+        <v>5192.368434301948</v>
+      </c>
+      <c r="Z121" t="n">
         <v>30</v>
       </c>
-      <c r="V121" t="n">
+      <c r="AA121" t="n">
         <v>30</v>
       </c>
-      <c r="W121" t="inlineStr">
+      <c r="AB121" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -12392,12 +14457,29 @@
         <v>7996</v>
       </c>
       <c r="U122" t="n">
+        <v>969.2121212121212</v>
+      </c>
+      <c r="V122" t="n">
+        <v>5185.284848484848</v>
+      </c>
+      <c r="W122" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X122" t="n">
+        <v>0.9099162135155621</v>
+      </c>
+      <c r="Y122" t="n">
+        <v>5184.374932271333</v>
+      </c>
+      <c r="Z122" t="n">
         <v>25</v>
       </c>
-      <c r="V122" t="n">
+      <c r="AA122" t="n">
         <v>25</v>
       </c>
-      <c r="W122" t="inlineStr">
+      <c r="AB122" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -12490,12 +14572,29 @@
         <v>7996</v>
       </c>
       <c r="U123" t="n">
-        <v>15</v>
+        <v>888.4444444444445</v>
       </c>
       <c r="V123" t="n">
-        <v>15</v>
+        <v>5152.977777777777</v>
       </c>
       <c r="W123" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X123" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y123" t="n">
+        <v>5152.507453645388</v>
+      </c>
+      <c r="Z123" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA123" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB123" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -12588,12 +14687,29 @@
         <v>7950</v>
       </c>
       <c r="U124" t="n">
+        <v>935.2941176470588</v>
+      </c>
+      <c r="V124" t="n">
+        <v>5144.117647058823</v>
+      </c>
+      <c r="W124" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X124" t="n">
+        <v>0.9099162135155621</v>
+      </c>
+      <c r="Y124" t="n">
+        <v>5143.207730845308</v>
+      </c>
+      <c r="Z124" t="n">
         <v>18</v>
       </c>
-      <c r="V124" t="n">
+      <c r="AA124" t="n">
         <v>18</v>
       </c>
-      <c r="W124" t="inlineStr">
+      <c r="AB124" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -12686,12 +14802,29 @@
         <v>7845</v>
       </c>
       <c r="U125" t="n">
-        <v>15</v>
+        <v>950.9090909090909</v>
       </c>
       <c r="V125" t="n">
-        <v>15</v>
+        <v>5087.363636363636</v>
       </c>
       <c r="W125" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X125" t="n">
+        <v>0.9099162135155621</v>
+      </c>
+      <c r="Y125" t="n">
+        <v>5086.453720150121</v>
+      </c>
+      <c r="Z125" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA125" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB125" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -12784,12 +14917,29 @@
         <v>7845</v>
       </c>
       <c r="U126" t="n">
-        <v>15</v>
+        <v>932.0792079207921</v>
       </c>
       <c r="V126" t="n">
-        <v>15</v>
+        <v>5079.831683168317</v>
       </c>
       <c r="W126" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X126" t="n">
+        <v>0.9099162135155621</v>
+      </c>
+      <c r="Y126" t="n">
+        <v>5078.921766954802</v>
+      </c>
+      <c r="Z126" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA126" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB126" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -12882,12 +15032,29 @@
         <v>7845</v>
       </c>
       <c r="U127" t="n">
-        <v>15</v>
+        <v>871.6666666666666</v>
       </c>
       <c r="V127" t="n">
-        <v>15</v>
+        <v>5055.666666666667</v>
       </c>
       <c r="W127" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X127" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y127" t="n">
+        <v>5055.196342534277</v>
+      </c>
+      <c r="Z127" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA127" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB127" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -12980,12 +15147,29 @@
         <v>7740</v>
       </c>
       <c r="U128" t="n">
+        <v>860</v>
+      </c>
+      <c r="V128" t="n">
+        <v>4988</v>
+      </c>
+      <c r="W128" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X128" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y128" t="n">
+        <v>4987.52967586761</v>
+      </c>
+      <c r="Z128" t="n">
         <v>6</v>
       </c>
-      <c r="V128" t="n">
+      <c r="AA128" t="n">
         <v>6</v>
       </c>
-      <c r="W128" t="inlineStr">
+      <c r="AB128" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -13078,12 +15262,29 @@
         <v>7652</v>
       </c>
       <c r="U129" t="n">
-        <v>15</v>
+        <v>900.2352941176471</v>
       </c>
       <c r="V129" t="n">
-        <v>15</v>
+        <v>4951.294117647059</v>
       </c>
       <c r="W129" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X129" t="n">
+        <v>0.9099162135155621</v>
+      </c>
+      <c r="Y129" t="n">
+        <v>4950.384201433543</v>
+      </c>
+      <c r="Z129" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA129" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB129" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -13176,12 +15377,29 @@
         <v>7652</v>
       </c>
       <c r="U130" t="n">
-        <v>15</v>
+        <v>956.5</v>
       </c>
       <c r="V130" t="n">
-        <v>15</v>
+        <v>4973.8</v>
       </c>
       <c r="W130" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X130" t="n">
+        <v>0.9099162135155621</v>
+      </c>
+      <c r="Y130" t="n">
+        <v>4972.890083786485</v>
+      </c>
+      <c r="Z130" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA130" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB130" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -13274,12 +15492,29 @@
         <v>7652</v>
       </c>
       <c r="U131" t="n">
+        <v>900.2352941176471</v>
+      </c>
+      <c r="V131" t="n">
+        <v>4951.294117647059</v>
+      </c>
+      <c r="W131" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X131" t="n">
+        <v>0.9099162135155621</v>
+      </c>
+      <c r="Y131" t="n">
+        <v>4950.384201433543</v>
+      </c>
+      <c r="Z131" t="n">
         <v>12</v>
       </c>
-      <c r="V131" t="n">
+      <c r="AA131" t="n">
         <v>12</v>
       </c>
-      <c r="W131" t="inlineStr">
+      <c r="AB131" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -13372,12 +15607,29 @@
         <v>7652</v>
       </c>
       <c r="U132" t="n">
-        <v>15</v>
+        <v>900.2352941176471</v>
       </c>
       <c r="V132" t="n">
-        <v>15</v>
+        <v>4951.294117647059</v>
       </c>
       <c r="W132" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X132" t="n">
+        <v>0.9099162135155621</v>
+      </c>
+      <c r="Y132" t="n">
+        <v>4950.384201433543</v>
+      </c>
+      <c r="Z132" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA132" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB132" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -13470,12 +15722,29 @@
         <v>7652</v>
       </c>
       <c r="U133" t="n">
-        <v>15</v>
+        <v>900.2352941176471</v>
       </c>
       <c r="V133" t="n">
-        <v>15</v>
+        <v>4951.294117647059</v>
       </c>
       <c r="W133" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X133" t="n">
+        <v>0.9099162135155621</v>
+      </c>
+      <c r="Y133" t="n">
+        <v>4950.384201433543</v>
+      </c>
+      <c r="Z133" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA133" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB133" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -13568,12 +15837,29 @@
         <v>7652</v>
       </c>
       <c r="U134" t="n">
-        <v>15</v>
+        <v>805.4736842105264</v>
       </c>
       <c r="V134" t="n">
-        <v>15</v>
+        <v>4913.38947368421</v>
       </c>
       <c r="W134" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X134" t="n">
+        <v>0.4703241323893724</v>
+      </c>
+      <c r="Y134" t="n">
+        <v>4912.919149551821</v>
+      </c>
+      <c r="Z134" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA134" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB134" t="inlineStr">
         <is>
           <t>16/01/2026</t>
         </is>
@@ -13666,12 +15952,29 @@
         <v>3698</v>
       </c>
       <c r="U135" t="n">
+        <v>410.8888888888889</v>
+      </c>
+      <c r="V135" t="n">
+        <v>2383.155555555555</v>
+      </c>
+      <c r="W135" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X135" t="n">
+        <v>0.4493598410330986</v>
+      </c>
+      <c r="Y135" t="n">
+        <v>2382.706195714522</v>
+      </c>
+      <c r="Z135" t="n">
         <v>19</v>
       </c>
-      <c r="V135" t="n">
+      <c r="AA135" t="n">
         <v>7</v>
       </c>
-      <c r="W135" t="inlineStr">
+      <c r="AB135" t="inlineStr">
         <is>
           <t>17/01/2026</t>
         </is>
@@ -13764,12 +16067,29 @@
         <v>3698</v>
       </c>
       <c r="U136" t="n">
+        <v>448.2424242424242</v>
+      </c>
+      <c r="V136" t="n">
+        <v>2398.09696969697</v>
+      </c>
+      <c r="W136" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X136" t="n">
+        <v>0.9009529739402599</v>
+      </c>
+      <c r="Y136" t="n">
+        <v>2397.19601672303</v>
+      </c>
+      <c r="Z136" t="n">
         <v>30</v>
       </c>
-      <c r="V136" t="n">
-        <v>0</v>
-      </c>
-      <c r="W136" t="inlineStr">
+      <c r="AA136" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB136" t="inlineStr">
         <is>
           <t>17/01/2026</t>
         </is>
@@ -13862,12 +16182,29 @@
         <v>3698</v>
       </c>
       <c r="U137" t="n">
-        <v>15</v>
+        <v>435.0588235294118</v>
       </c>
       <c r="V137" t="n">
-        <v>0</v>
+        <v>2392.823529411764</v>
       </c>
       <c r="W137" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X137" t="n">
+        <v>0.9009529739402599</v>
+      </c>
+      <c r="Y137" t="n">
+        <v>2391.922576437824</v>
+      </c>
+      <c r="Z137" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA137" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB137" t="inlineStr">
         <is>
           <t>17/01/2026</t>
         </is>
@@ -13960,12 +16297,29 @@
         <v>3698</v>
       </c>
       <c r="U138" t="n">
-        <v>15</v>
+        <v>462.25</v>
       </c>
       <c r="V138" t="n">
-        <v>0</v>
+        <v>2403.7</v>
       </c>
       <c r="W138" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X138" t="n">
+        <v>0.9009529739402599</v>
+      </c>
+      <c r="Y138" t="n">
+        <v>2402.79904702606</v>
+      </c>
+      <c r="Z138" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA138" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB138" t="inlineStr">
         <is>
           <t>17/01/2026</t>
         </is>
@@ -14058,12 +16412,29 @@
         <v>3698</v>
       </c>
       <c r="U139" t="n">
+        <v>457.4845360824742</v>
+      </c>
+      <c r="V139" t="n">
+        <v>2401.79381443299</v>
+      </c>
+      <c r="W139" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X139" t="n">
+        <v>0.9009529739402599</v>
+      </c>
+      <c r="Y139" t="n">
+        <v>2400.89286145905</v>
+      </c>
+      <c r="Z139" t="n">
         <v>30</v>
       </c>
-      <c r="V139" t="n">
-        <v>0</v>
-      </c>
-      <c r="W139" t="inlineStr">
+      <c r="AA139" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB139" t="inlineStr">
         <is>
           <t>17/01/2026</t>
         </is>
@@ -14156,12 +16527,29 @@
         <v>3698</v>
       </c>
       <c r="U140" t="n">
+        <v>448.2424242424242</v>
+      </c>
+      <c r="V140" t="n">
+        <v>2398.09696969697</v>
+      </c>
+      <c r="W140" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X140" t="n">
+        <v>0.9009529739402599</v>
+      </c>
+      <c r="Y140" t="n">
+        <v>2397.19601672303</v>
+      </c>
+      <c r="Z140" t="n">
         <v>30</v>
       </c>
-      <c r="V140" t="n">
-        <v>0</v>
-      </c>
-      <c r="W140" t="inlineStr">
+      <c r="AA140" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB140" t="inlineStr">
         <is>
           <t>17/01/2026</t>
         </is>
@@ -14254,12 +16642,29 @@
         <v>3698</v>
       </c>
       <c r="U141" t="n">
+        <v>457.4845360824742</v>
+      </c>
+      <c r="V141" t="n">
+        <v>2401.79381443299</v>
+      </c>
+      <c r="W141" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X141" t="n">
+        <v>0.9009529739402599</v>
+      </c>
+      <c r="Y141" t="n">
+        <v>2400.89286145905</v>
+      </c>
+      <c r="Z141" t="n">
         <v>30</v>
       </c>
-      <c r="V141" t="n">
-        <v>0</v>
-      </c>
-      <c r="W141" t="inlineStr">
+      <c r="AA141" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB141" t="inlineStr">
         <is>
           <t>17/01/2026</t>
         </is>
@@ -14352,12 +16757,29 @@
         <v>3698</v>
       </c>
       <c r="U142" t="n">
-        <v>15</v>
+        <v>410.8888888888889</v>
       </c>
       <c r="V142" t="n">
-        <v>0</v>
+        <v>2383.155555555555</v>
       </c>
       <c r="W142" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X142" t="n">
+        <v>0.4493598410330986</v>
+      </c>
+      <c r="Y142" t="n">
+        <v>2382.706195714522</v>
+      </c>
+      <c r="Z142" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA142" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB142" t="inlineStr">
         <is>
           <t>17/01/2026</t>
         </is>
@@ -14450,12 +16872,29 @@
         <v>3494</v>
       </c>
       <c r="U143" t="n">
+        <v>436.75</v>
+      </c>
+      <c r="V143" t="n">
+        <v>2271.1</v>
+      </c>
+      <c r="W143" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X143" t="n">
+        <v>0.9009529739402599</v>
+      </c>
+      <c r="Y143" t="n">
+        <v>2270.19904702606</v>
+      </c>
+      <c r="Z143" t="n">
         <v>4</v>
       </c>
-      <c r="V143" t="n">
-        <v>0</v>
-      </c>
-      <c r="W143" t="inlineStr">
+      <c r="AA143" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB143" t="inlineStr">
         <is>
           <t>17/01/2026</t>
         </is>
@@ -14548,12 +16987,29 @@
         <v>3302</v>
       </c>
       <c r="U144" t="n">
+        <v>412.75</v>
+      </c>
+      <c r="V144" t="n">
+        <v>2146.3</v>
+      </c>
+      <c r="W144" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X144" t="n">
+        <v>0.9009529739402599</v>
+      </c>
+      <c r="Y144" t="n">
+        <v>2145.39904702606</v>
+      </c>
+      <c r="Z144" t="n">
         <v>10</v>
       </c>
-      <c r="V144" t="n">
-        <v>0</v>
-      </c>
-      <c r="W144" t="inlineStr">
+      <c r="AA144" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB144" t="inlineStr">
         <is>
           <t>17/01/2026</t>
         </is>
@@ -14646,12 +17102,29 @@
         <v>3296</v>
       </c>
       <c r="U145" t="n">
+        <v>412</v>
+      </c>
+      <c r="V145" t="n">
+        <v>2142.4</v>
+      </c>
+      <c r="W145" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X145" t="n">
+        <v>0.9009529739402599</v>
+      </c>
+      <c r="Y145" t="n">
+        <v>2141.49904702606</v>
+      </c>
+      <c r="Z145" t="n">
         <v>7</v>
       </c>
-      <c r="V145" t="n">
-        <v>0</v>
-      </c>
-      <c r="W145" t="inlineStr">
+      <c r="AA145" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB145" t="inlineStr">
         <is>
           <t>17/01/2026</t>
         </is>
@@ -14744,12 +17217,29 @@
         <v>3288</v>
       </c>
       <c r="U146" t="n">
+        <v>411</v>
+      </c>
+      <c r="V146" t="n">
+        <v>2137.2</v>
+      </c>
+      <c r="W146" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X146" t="n">
+        <v>0.9009529739402599</v>
+      </c>
+      <c r="Y146" t="n">
+        <v>2136.29904702606</v>
+      </c>
+      <c r="Z146" t="n">
         <v>3</v>
       </c>
-      <c r="V146" t="n">
-        <v>0</v>
-      </c>
-      <c r="W146" t="inlineStr">
+      <c r="AA146" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB146" t="inlineStr">
         <is>
           <t>17/01/2026</t>
         </is>
@@ -14842,12 +17332,29 @@
         <v>752</v>
       </c>
       <c r="U147" t="n">
+        <v>93.03092783505154</v>
+      </c>
+      <c r="V147" t="n">
+        <v>488.4123711340206</v>
+      </c>
+      <c r="W147" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X147" t="n">
+        <v>0.9063949250523571</v>
+      </c>
+      <c r="Y147" t="n">
+        <v>487.5059762089682</v>
+      </c>
+      <c r="Z147" t="n">
         <v>11</v>
       </c>
-      <c r="V147" t="n">
-        <v>0</v>
-      </c>
-      <c r="W147" t="inlineStr">
+      <c r="AA147" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB147" t="inlineStr">
         <is>
           <t>18/01/2026</t>
         </is>
@@ -14940,12 +17447,29 @@
         <v>752</v>
       </c>
       <c r="U148" t="n">
-        <v>15</v>
+        <v>94</v>
       </c>
       <c r="V148" t="n">
-        <v>0</v>
+        <v>488.8</v>
       </c>
       <c r="W148" t="inlineStr">
+        <is>
+          <t>8_9</t>
+        </is>
+      </c>
+      <c r="X148" t="n">
+        <v>0.9063949250523571</v>
+      </c>
+      <c r="Y148" t="n">
+        <v>487.8936050749476</v>
+      </c>
+      <c r="Z148" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA148" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB148" t="inlineStr">
         <is>
           <t>18/01/2026</t>
         </is>
@@ -15038,12 +17562,29 @@
         <v>752</v>
       </c>
       <c r="U149" t="n">
-        <v>15</v>
+        <v>83.55555555555556</v>
       </c>
       <c r="V149" t="n">
-        <v>0</v>
+        <v>484.6222222222222</v>
       </c>
       <c r="W149" t="inlineStr">
+        <is>
+          <t>ge9</t>
+        </is>
+      </c>
+      <c r="X149" t="n">
+        <v>0.4493598410330986</v>
+      </c>
+      <c r="Y149" t="n">
+        <v>484.1728623811891</v>
+      </c>
+      <c r="Z149" t="n">
+        <v>15</v>
+      </c>
+      <c r="AA149" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB149" t="inlineStr">
         <is>
           <t>18/01/2026</t>
         </is>
@@ -15136,12 +17677,29 @@
         <v>670</v>
       </c>
       <c r="U150" t="n">
+        <v>89.33333333333333</v>
+      </c>
+      <c r="V150" t="n">
+        <v>437.7333333333333</v>
+      </c>
+      <c r="W150" t="inlineStr">
+        <is>
+          <t>7_8</t>
+        </is>
+      </c>
+      <c r="X150" t="n">
+        <v>0.6190701577567638</v>
+      </c>
+      <c r="Y150" t="n">
+        <v>437.1142631755766</v>
+      </c>
+      <c r="Z150" t="n">
         <v>1</v>
       </c>
-      <c r="V150" t="n">
-        <v>0</v>
-      </c>
-      <c r="W150" t="inlineStr">
+      <c r="AA150" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB150" t="inlineStr">
         <is>
           <t>18/01/2026</t>
         </is>

</xml_diff>